<commit_message>
fix(review): cột văn bản tác động của phiếu gold độc lập dễ đọc
Mỗi văn bản một dòng, gộp quan hệ trùng, chỉ ghi số hiệu, thêm ngày hiệu
lực (từ bản crawl, hoặc index theo số hiệu), xếp theo thời gian; VBHN ghi
"chỉ để tham khảo lời văn" và xếp cuối. Chưa ai điền phiếu nên xuất lại an
toàn; thông tin thêm là dữ liệu cổng, không phải đáp án của đồ thị.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/gold_A.xlsx
+++ b/data/review/gold_A.xlsx
@@ -712,7 +712,8 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Thông tư số 07/2024/TT-BKHCN Sửa đổi, bổ sung một số điều tại các văn bản quy phạm pháp luật thuộc thẩm quyền của Bộ trưởng Bộ Khoa học và C (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170642)</t>
+          <t>• 07/2024/TT-BKHCN — sửa đổi, bổ sung — hiệu lực 22/11/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170642</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr"/>
@@ -754,7 +755,8 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 88/2025/NĐ-CP Quy định chi tiết và hướng dẫn một số điều của Nghị quyết số 193/2025/QH15 ngày 19 tháng 02 năm 2025 của Quốc hội (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=177799)</t>
+          <t>• 88/2025/NĐ-CP — bãi bỏ — hiệu lực 13/04/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=177799</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr"/>
@@ -796,7 +798,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 56/2019/TT-BTC Sửa đổi, bổ sung một số điều của Thông tư số 49/2015/TT-BTC ngày 14 tháng 4 năm 2015 quy định thủ tục hải quan đố (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137595) | hợp nhất: Văn bản hợp nhất số 01/VBHN-BTC Thông tư quy định thủ tục hải quan đối với hàng hóa xuất khẩu, nhập khẩu, quá cảnh gửi qua dịch vụ chuyển ph (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=140467) | sửa đổi, bổ sung: Thông tư số 56/2019/TT-BTC Sửa đổi, bổ sung một số điều của Thông tư số 49/2015/TT-BTC ngày 14 tháng 4 năm 2015 quy định thủ tục hải quan đố (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137595) | sửa đổi, bổ sung: Thông tư số 29/2025/TT-BTC Sửa đổi, bổ sung một số điều của Thông tư số 191/2015/TT-BTC ngày 24 tháng 11 năm 2015 quy định thủ tục hải quan  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178369)</t>
+          <t>• 56/2019/TT-BTC — bãi bỏ, sửa đổi, bổ sung — hiệu lực 15/10/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137595
+• 29/2025/TT-BTC — sửa đổi, bổ sung — hiệu lực 09/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178369
+• 01/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=140467</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr"/>
@@ -838,7 +845,10 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 10/VBHN-BTC Hướng dẫn việc chuyển giao quyền đại diện chủ sở hữu nhà nước tại Tổng công ty Đầu tư và Kinh doanh vốn Nhà  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=157328) | sửa đổi, bổ sung: Thông tư số 119/2021/TT-BTC Sửa đổi, bổ sung một số Điều của Thông tư số 83/2018/TT-BTC ngày 30 tháng 08 năm 2018 của Bộ trưởng Bộ Tài chính (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152520)</t>
+          <t>• 119/2021/TT-BTC — sửa đổi, bổ sung — hiệu lực 15/02/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152520
+• 10/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=157328</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr"/>
@@ -880,7 +890,8 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Nghị định số 84/2026/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định của Chính phủ trong lĩnh vực quản lý nợ công (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187842)</t>
+          <t>• 84/2026/NĐ-CP — sửa đổi, bổ sung — hiệu lực 25/03/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187842</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
@@ -922,7 +933,28 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 100/2018/NĐ-CP Sửa đổi, bổ sung, bãi bỏ một số quy định về điều kiện đầu tư kinh doanh thuộc các lĩnh vực quản lý nhà n (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=130011) | bãi bỏ: Nghị định số 96/2024/NĐ-CP Quy định chi tiết một số điều của Luật Kinh doanh bất động sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169708) | bãi bỏ: Nghị định số 207/2026/NĐ-CP Quy định chi tiết một số điều của Luật Xây dựng về quản lý chất lượng, thi công xây dựng và bảo trì công trình x (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=c4911dc0-6e5b-11f1-b871-73e465f01c71) | bãi bỏ: Nghị định số 35/2026/NĐ-CP Quy định chi tiết một số điều của Nghị quyết về phân loại đô thị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186907) | hợp nhất: Văn bản hợp nhất số 15/VBHN-BXD Nghị định về quản lý đầu tư phát triển đô thị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162924) | hợp nhất: Văn bản hợp nhất số 03/VBHN-BXD Nghị định về quản lý đầu tư phát triển đô thị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160736) | hợp nhất: Văn bản hợp nhất số 07/VBHN-BXD NGhị định về quản lý đầu tư phát triển đô thị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=131170) | hợp nhất: Văn bản hợp nhất số 07/VBHN-BXD NGhị định về quản lý đầu tư phát triển đô thị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=131171) | hợp nhất: Văn bản hợp nhất số 04/VBHN-BXD Nghị định về quản lý đầu tư phát triển đô thị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=171791) | sửa đổi, bổ sung: Nghị định số 31/2021/NĐ-CP Quy định chi tiết và hướng dẫn thi hành một số điều của Luật Đầu tư (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147720) | sửa đổi, bổ sung: Nghị định số 35/2023/NĐ-CP sửa đổi, bổ sung một số điều của các Nghị định thuộc lĩnh vực quản lý nhà nước của Bộ Xây dựng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160908)</t>
+          <t>• 100/2018/NĐ-CP — bãi bỏ — hiệu lực 15/09/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=130011
+• 31/2021/NĐ-CP — sửa đổi, bổ sung — hiệu lực 26/03/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147720
+• 35/2023/NĐ-CP — sửa đổi, bổ sung — hiệu lực 20/06/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160908
+• 96/2024/NĐ-CP — bãi bỏ — hiệu lực 01/08/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169708
+• 35/2026/NĐ-CP — bãi bỏ — hiệu lực 22/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186907
+• 207/2026/NĐ-CP — bãi bỏ — hiệu lực 01/07/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=c4911dc0-6e5b-11f1-b871-73e465f01c71
+• 03/VBHN-BXD — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160736
+• 04/VBHN-BXD — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=171791
+• 07/VBHN-BXD — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=131170
+• 07/VBHN-BXD — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=131171
+• 15/VBHN-BXD — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162924</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr"/>
@@ -964,7 +996,10 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 03/VBHN-BTC Hướng dẫn về phí và lệ phí thuộc thẩm quyền quyết định của Hội đồng nhân dân tỉnh, thành phố trực thuộc trun (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=156563) | sửa đổi, bổ sung: Thông tư số 106/2021/TT-BTC Sửa đổi, bổ sung một số điều của Thông tư số 85/2019/TT-BTC ngày 29 tháng 11 năm 2019 của Bộ trưởng Bộ Tài chính (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152278)</t>
+          <t>• 106/2021/TT-BTC — sửa đổi, bổ sung — hiệu lực 10/01/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152278
+• 03/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=156563</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr"/>
@@ -1006,7 +1041,28 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 41/2026/TT-BCT Quy định Danh mục phế liệu và Danh mục hàng hóa đã qua sử dụng tạm ngừng kinh doanh tạm nhập, tái xuất, chuyển kh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=bccbb3d0-873c-11f1-82a9-63ca2e29bb67) | hợp nhất: Văn bản hợp nhất số 29/VBHN-BCT Thông tư Quy định chi tiết một số điều của Luật Quản lý ngoại thương và Nghị định số 69/2018/NĐ-CP ngày 15 t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179760) | hợp nhất: Văn bản hợp nhất số 06/VBHN-BCT Quy định chi tiết một số điều của Luật Quản lý ngoại thương và Nghị định số 69/2018/NĐ-CP ngày 15 tháng 5 nă (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141174) | hợp nhất: Văn bản hợp nhất số 11/VBHN-BCT Thông tư bổ sung Danh mục chi tiết theo mã số HS của hàng hóa xuất khẩu, nhập khẩu quy định tại một số Thông (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160168) | hợp nhất: Văn bản hợp nhất số 24/VBHN-BCT Thông tư quy định chi tiết một số điều của Luật Quản lý ngoại thương và Nghị định số 69/2018/NĐ-CP ngày 15 t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=8ad6daf0-7f6f-11f1-9e1f-cba12064fd97) | hợp nhất: Văn bản hợp nhất số 47/VBHN-BCT Thông tư quy định chi tiết một số điều của Luật Quản lý ngoại thương và Nghị định số 69/2018/NĐ-CP ngày 15 t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=14214f70-6891-11f1-801e-4db6a607ef12) | hợp nhất: Văn bản hợp nhất số 70/2026/VBHN-TT-BCT Thông tư quy định chi tiết một số điều của Luật Quản lý ngoại thương và Nghị định số 69/2018/NĐ-CP n (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=d7e65af0-926b-11f1-a5a9-cb03c709c8ec) | sửa đổi, bổ sung: Thông tư 26/2026/TT-BCT Sửa đổi, bổ sung một số quy định về phân cấp, cắt giảm, đơn giản hóa thủ tục hành chính trong các lĩnh vực thuộc phạ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=c38d4c80-5819-11f1-8cfa-090ca3b5a55f) | sửa đổi, bổ sung: Thông tư số 38/2025/TT-BCT sửa đổi, bổ sung một số quy định về phân cấp thực hiện thủ tục hành chính trong các lĩnh vực thuộc phạm vi quản l (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178549) | sửa đổi, bổ sung: Thông tư số 08/2023/TT-BCT sửa đổi, bổ sung một số điều quy định Danh mục chi tiết theo mã số HS của hàng hóa xuất khẩu, nhập khẩu ban hành  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160072) | sửa đổi, bổ sung: Thông tư số 42/2019/TT-BCT Sửa đổi, bổ sung một số quy định về chế độ báo cáo định kỳ tại các Thông tư do Bộ trưởng Bộ Công Thương ban hành  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139672)</t>
+          <t>• 42/2019/TT-BCT — sửa đổi, bổ sung — hiệu lực 05/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139672
+• 08/2023/TT-BCT — sửa đổi, bổ sung — hiệu lực 16/05/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160072
+• 38/2025/TT-BCT — sửa đổi, bổ sung — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178549
+• Thông tư 26/2026/TT-BCT Sửa đổi, bổ sung một số quy định về phân cấp, cắt giảm, đơn giản h — sửa đổi, bổ sung — hiệu lực 29/05/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=c38d4c80-5819-11f1-8cfa-090ca3b5a55f
+• 41/2026/TT-BCT — bãi bỏ — hiệu lực 05/09/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=bccbb3d0-873c-11f1-82a9-63ca2e29bb67
+• 06/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141174
+• 11/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160168
+• 24/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=8ad6daf0-7f6f-11f1-9e1f-cba12064fd97
+• 29/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179760
+• 47/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=14214f70-6891-11f1-801e-4db6a607ef12
+• 70/2026/VBHN-TT-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=d7e65af0-926b-11f1-a5a9-cb03c709c8ec</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr"/>
@@ -1048,7 +1104,14 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Nghị định số 55/2023/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 75/2021/NĐ-CP ngày 24/7/2021 quy định mức hưởng trợ cấp, phụ cấp và (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169616) | sửa đổi, bổ sung: Nghị định số 77/2024/NĐ-C Sửa đổi, bổ sung một số điều của Nghị định số 75/2021/NĐ-CP ngày 24 tháng 7 năm 2021 của Chính phủ quy định mức hư (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=173646) | thay thế: Nghị định số 321/2026/NĐ-CP quy định mức hưởng trợ cấp, phụ cấp và các chế độ ưu đãi người có công với cách mạng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=5bfb4a00-9c83-11f1-9722-67b318d484b4) | thay thế: Nghị quyết số 26/2026/NQ-CP Về cơ chế, chính sách đặc thù nhằm tháo gỡ khó khăn trong tổ chức lấy mẫu, giám định và xác định danh tính hài c (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=539a1450-7a13-11f1-bfab-2d6d51f414a0)</t>
+          <t>• 55/2023/NĐ-CP — sửa đổi, bổ sung — hiệu lực 05/09/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169616
+• 77/2024/NĐ-C — sửa đổi, bổ sung — hiệu lực 01/07/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=173646
+• 26/2026/NQ-CP — thay thế — hiệu lực 06/05/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=539a1450-7a13-11f1-bfab-2d6d51f414a0
+• 321/2026/NĐ-CP — thay thế — hiệu lực 01/10/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=5bfb4a00-9c83-11f1-9722-67b318d484b4</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr"/>
@@ -1090,7 +1153,8 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>thay thế: Thông tư số 45/2009/TT-BCA(C11) Hướng dẫn thi hành một số điều của Nghị định số 52/2008/NĐ-CP ngày 22 tháng 4 năm 2008 về quản lý kinh doanh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=11741)</t>
+          <t>• 45/2009/TT-BCA(C11) — thay thế — hiệu lực 28/08/2009
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=11741</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr"/>
@@ -1132,7 +1196,22 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 92/2023/NĐ-CP Bãi bỏ một số văn bản quy phạm pháp luật của Chính phủ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164308) | hợp nhất: Văn bản hợp nhất số 951/VBHN-BTP Quy định chi tiết thi hành một số điều của Luật nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134587) | hợp nhất: Văn bản hợp nhất số 275/VBHN-BTP Quy định chi tiết thi hành một số điều của Luật Nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174653) | sửa đổi, bổ sung: Nghị định số 24/2019/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 19/2011/NĐ-CP ngày 21 tháng 3 năm 2011 của Chính phủ quy định chi t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134536) | sửa đổi, bổ sung: Nghị định số 18/2026/NĐ-CP Sửa đổi, bổ sung một số nghị định để cắt giảm, đơn giản hóa thủ tục hành chính, điều kiện kinh doanh thuộc phạm v (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187582) | sửa đổi, bổ sung: Nghị định số 06/2025/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định về nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174313) | sửa đổi, bổ sung: Nghị định số 114/2016/NĐ-CP Quy định lệ phí đăng ký nuôi con nuôi, lệ phí cấp giấy phép hoạt động của tổ chức con nuôi nước ngoài (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112160) | sửa đổi, bổ sung: Nghị định số 104/2022/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định liên quan đến việc nộp, xuất trình sổ hộ khẩu, sổ tạm trú giấy kh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167220)</t>
+          <t>• 114/2016/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112160
+• 24/2019/NĐ-CP — sửa đổi, bổ sung — hiệu lực 25/04/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134536
+• 104/2022/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167220
+• 92/2023/NĐ-CP — bãi bỏ — hiệu lực 19/12/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164308
+• 06/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 08/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174313
+• 18/2026/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187582
+• 275/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174653
+• 951/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134587</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr"/>
@@ -1174,7 +1253,8 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Thông tư số 15/2018/TT-BTC Quy định về chi phí phát hành, hoán đểi, mua lại, thanh toán gốc, lãi trái phiếu Chính phủ, trái phiếu đuọc Chính (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=128189)</t>
+          <t>• 15/2018/TT-BTC — sửa đổi, bổ sung — hiệu lực 01/04/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=128189</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr"/>
@@ -1216,7 +1296,14 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 156/2025/TT-BTC Sửa đổi, bổ sung một số điều của Thông tư số 199/2016/TT-BTC ngày 08 tháng 11 năm 2016 của Bộ trưởng Bộ Tài chín (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186182) | bãi bỏ: Thông tư 30/2026/TT-BTC Quy định mức thu, chế độ thu, nộp phí thẩm định cấp giấy phép hoạt động điện lực (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=f9b4a860-5a3c-11f1-9b9f-173bd8f4ab4f) | bãi bỏ: Thông tư số 11/2026/TT-BTС Quy định mức thu, chế độ thu, nộp phí thuộc lĩnh vực đường sắt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186990) | sửa đổi, bổ sung: Thông tư 11/2026/TT-BTC Quy định mức thu, chế độ thu, nộp phí thuộc lĩnh vực đường sắt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=bf3acd10-599f-11f1-bcbf-37bff26920b0) | sửa đổi, bổ sung: Thông tư số 11/2026/TT-BTС Quy định mức thu, chế độ thu, nộp phí thuộc lĩnh vực đường sắt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186990)</t>
+          <t>• 156/2025/TT-BTC — bãi bỏ — hiệu lực 01/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186182
+• 11/2026/TT-BTС — bãi bỏ, sửa đổi, bổ sung — hiệu lực 27/03/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186990
+• Thông tư 11/2026/TT-BTC Quy định mức thu, chế độ thu, nộp phí thuộc lĩnh vực đường sắt — sửa đổi, bổ sung — hiệu lực 27/03/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=bf3acd10-599f-11f1-bcbf-37bff26920b0
+• Thông tư 30/2026/TT-BTC Quy định mức thu, chế độ thu, nộp phí thẩm định cấp giấy phép hoạt — bãi bỏ — hiệu lực 11/05/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=f9b4a860-5a3c-11f1-9b9f-173bd8f4ab4f</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr"/>
@@ -1258,7 +1345,8 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Thông tư số 56/2023/TT-BGTVT Sửa đổi, bổ sung một số Điều của Thông tư số 23/2017/TT-BGTVT ngày 28 tháng 07 năm 2017 của Bộ trưởng Bộ Giao t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=165446)</t>
+          <t>• 56/2023/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 01/04/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=165446</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr"/>
@@ -1300,7 +1388,32 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 07/VBHN-NHNN Quy định về giao nhận, bảo quản, vận chuyển tiền mặt, tài sản quý, giấy tờ có giá (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178572) | hợp nhất: Văn bản hợp nhất số 24/VBHN-NHNN Thông tư hướng dẫn việc tổ chức thực hiện hoạt động quản lý dự trữ ngoại hối nhà nước (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164720) | hợp nhất: Văn bản hợp nhất số 32/VBHN-NHNN Hướng dẫn việc tổ chức thực hiện hoạt động quản lý dự trữ ngoại hối nhà nước (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170802) | hợp nhất: Văn bản hợp nhất số 07/VBHN-NHNN Quy định về giao nhận, bảo quản, vận chuyển tiền mặt, tài sản quý, giấy tờ có giá (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179742) | hợp nhất: Văn bản hợp nhất số 08/VBHN-NHNN Quy định về giao nhận, bảo quản, vận chuyển tiền mặt, tài sản quý, giấy tờ có giá (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=127031) | hợp nhất: Văn bản hợp nhất số 26/VBHN-NHNN Quy định về giao nhận, bảo quản, vận chuyển tiền mặt, tài sản quý, giấy tờ có giá (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=138098) | hợp nhất: Văn bản hợp nhất số 14/VBHN-NHNN Quy định về giao nhận, bảo quản, vận chuyển tiền mặt, tài sản quý, giấy tờ có giá (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=151816) | sửa đổi, bổ sung: Thông tư số 12/2023/TT-NHNN Sửa đổi, bổ sung một số điều của các văn bản quy phạm pháp luật quy định về việc triển khai nhiệm vụ quản lý dự  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162635) | sửa đổi, bổ sung: Thông tư số 19/2021/TT-NHNN Sửa đổi, bổ sung một số điều của Thông tư số 01/2014/TT-NHNN ngày 06/01/2014 của Thống đốc Ngân hàng Nhà nước Vi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=150860) | sửa đổi, bổ sung: Thông tư số 43/2024/TT-NHNN sửa đổi, bổ sung một số điều của Thông tư số 01/2014/TT-NHNN ngày 10 tháng 12 năm 2014 của Thống đốc Ngân hàng N (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169221) | sửa đổi, bổ sung: Thông tư số 14/2019/TT-NHNN Sửa đổi, bổ sung một số điều tại các Thông tư có quy định về chế độ báo cáo định kỳ của Ngân hàng Nhà nước (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137583) | sửa đổi, bổ sung: Thông tư số 05/2025/TT-NHNN Sửa đổi, bổ sung một số điều của Thông tư số 01/2014/TT-NHNN ngày 06/01/2014 của Thống đốc Ngân hàng Nhà nước Vi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178168) | sửa đổi, bổ sung: Thông tư số 12/2017/TT-NHNN Sửa đổi, bổ sung một số điều của Thông tư số 01/2014/TT-NHNN ngày 06/01/2014 của Thống đốc Ngân hàng Nhà nước Vi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=124628)</t>
+          <t>• 12/2017/TT-NHNN — sửa đổi, bổ sung — hiệu lực 16/10/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=124628
+• 14/2019/TT-NHNN — sửa đổi, bổ sung — hiệu lực 15/10/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137583
+• 19/2021/TT-NHNN — sửa đổi, bổ sung — hiệu lực 08/01/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=150860
+• 12/2023/TT-NHNN — sửa đổi, bổ sung — hiệu lực 27/11/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162635
+• 43/2024/TT-NHNN — sửa đổi, bổ sung — hiệu lực 23/09/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169221
+• 05/2025/TT-NHNN — sửa đổi, bổ sung — hiệu lực 19/05/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178168
+• 07/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178572
+• 07/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179742
+• 08/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=127031
+• 14/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=151816
+• 24/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164720
+• 26/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=138098
+• 32/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170802</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr"/>
@@ -1342,7 +1455,10 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 25/2018/TT-BYT bãi bỏ một số văn bản quy phạm pháp luật trong lĩnh vực y tế Bộ trưởng Bộ Y tế ban hành, liên tịch ban hành (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137196) | bãi bỏ: Thông tư số 20/2023/TT-BYT Bãi bỏ một số văn bản quy phạm pháp luật do Bộ trưởng Bộ Y tế ban hành (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166212)</t>
+          <t>• 25/2018/TT-BYT — bãi bỏ — hiệu lực 15/11/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137196
+• 20/2023/TT-BYT — bãi bỏ — hiệu lực 01/01/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166212</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr"/>
@@ -1384,7 +1500,8 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 29/2018/TT-BCT Sửa đổi, bổ sung một số Thông tư quy định chế độ báo cáo định kỳ trong lĩnh vực Công Thương (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133197)</t>
+          <t>• 29/2018/TT-BCT — bãi bỏ — hiệu lực 12/11/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133197</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr"/>
@@ -1426,7 +1543,16 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 87/2015/TT-BGTVT Ban hành Quy chuẩn kỹ thuật quốc gia về chất lượng an toàn kỹ thuật và bảo vệ môi trường đối với xe ô tô (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111822) | bãi bỏ: Thông tư số 90/2015/TT-BGTVT Ban hành Quy chuẩn kỹ thuật quốc gia về chất lượng an toàn kỹ thuật và bảo vệ môi trường đối với ô tô khách thà (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111612) | bãi bỏ: Thông tư số 45/2023/TT-BGTVT Ban hành Quy chuẩn kỹ thuật quốc gia về chất lượng an toàn kỹ thuật và bảo vệ môi trường đối với xe máy chuyên  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164732) | bãi bỏ: Thông tư số 88/2015/TT-BGTVT Ban hành Quy chuẩn kỹ thuật quốc gia về chất lượng an toàn kỹ thuật đối với rơ moóc và sơ mi rơ moóc (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=98556) | bãi bỏ: Thông tư số 67/2015/TT-BGTVT Ban hành Quy chuẩn kỹ thuật quốc gia về chất lượng an toàn kỹ thuật và bảo vệ môi trường đối với xe mô tô, xe g (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111835)</t>
+          <t>• 67/2015/TT-BGTVT — bãi bỏ — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111835
+• 87/2015/TT-BGTVT — bãi bỏ — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111822
+• 88/2015/TT-BGTVT — bãi bỏ — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=98556
+• 90/2015/TT-BGTVT — bãi bỏ — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111612
+• 45/2023/TT-BGTVT — bãi bỏ — hiệu lực 01/07/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164732</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr"/>
@@ -1468,7 +1594,10 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 42/2019/TT-BCT Sửa đổi, bổ sung một số quy định về chế độ báo cáo định kỳ tại các Thông tư do Bộ trưởng Bộ Công Thương ban hành  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139672) | hợp nhất: Văn bản hợp nhất số 37/VBHN-BCT Ban hành Quy chuẩn kỹ thuật quốc gia đối với sản phẩm khăn giấy và giấy vệ sinh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141720)</t>
+          <t>• 42/2019/TT-BCT — bãi bỏ — hiệu lực 05/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139672
+• 37/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141720</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr"/>
@@ -1510,7 +1639,14 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 23/2024/TT-BTTTT bãi bỏ một số văn bản quy phạm pháp luật do Bộ trưởng Bộ Thông tin và Truyền thông ban hành hoặc liên tịch ban  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174567) | bãi bỏ: Thông tư số 23/2024/TT-BKHCN Bãi bỏ một số văn bản quy phạm pháp luật do Bộ trưởng Bộ Thông tin và Truyền thông ban hành hoặc liên tịch ban  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=184410) | sửa đổi, bổ sung: Thông tư số 10/2020/TT-BTTTT Sửa đổi, bổ sung một số nội dung của Thông tư số 30/2011/TT-BTTTT ngày 31 tháng 10 năm 2011 của Bộ trưởng Bộ Th (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=146204) | sửa đổi, bổ sung: Thông tư số 15/2018/TT-BTTTT Sửa đổi, bổ sung một số nội dung của Thông tư số 30/2011/TT-BTTTT ngày 31 tháng 10 năm 2011 của Bộ trưởng Bộ Th (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133255)</t>
+          <t>• 15/2018/TT-BTTTT — sửa đổi, bổ sung — hiệu lực 01/01/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133255
+• 10/2020/TT-BTTTT — sửa đổi, bổ sung — hiệu lực 01/07/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=146204
+• 23/2024/TT-BKHCN — bãi bỏ — hiệu lực 31/12/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=184410
+• 23/2024/TT-BTTTT — bãi bỏ — hiệu lực 31/12/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174567</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr"/>
@@ -1552,7 +1688,12 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 22/2016/TT-BXD Bãi bỏ toàn bộ hoặc một phần văn bản quy phạm pháp luật có quy định về điều kiện đầu tư kinh doanh do Bộ Xây dựng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112527) | sửa đổi, bổ sung: Thông tư số 06/2011/TT-BXD Sửa đổi Quy định về thủ tục hành chính trong lĩnh vực xây dựng; kiến trúc, quy hoạch xây dựng thực thi Nghị quyết (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=26668) | thay thế: Thông tư số 17/2016/TT-BXD Hướng dẫn về năng lực của tổ chức, cá nhân tham gia hoạt động xây dựng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111687)</t>
+          <t>• 06/2011/TT-BXD — sửa đổi, bổ sung — hiệu lực 05/08/2011
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=26668
+• 22/2016/TT-BXD — bãi bỏ — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112527
+• 17/2016/TT-BXD — thay thế — hiệu lực 01/09/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111687</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr"/>
@@ -1594,7 +1735,10 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 01/VBHN-BTTTT Quy định chi tiết và hướng dẫn thi hành một số điều của Luật Xuất bản và Nghị định số 195/2013/NĐ-CP ngày  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166347) | sửa đổi, bổ sung: Thông tư số 23/2023/TT-BTTTT Sửa đổi, bổ sung một số điều của Thông tư số 01/2020/TT-BTTTT ngày 07 tháng 02 năm 2020 của Bộ trưởng Bộ Thông  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166015)</t>
+          <t>• 23/2023/TT-BTTTT — sửa đổi, bổ sung — hiệu lực 07/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166015
+• 01/VBHN-BTTTT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166347</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr"/>
@@ -1636,7 +1780,12 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư 20/2026/TT-BTC Quy định chi tiết một số điều của Luật Thuế thu nhập doanh nghiệp và Nghị định số 320/2025/NĐ-CP ngày 15 tháng 12 nă (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=6fb7dd80-59a6-11f1-a013-532655e6581a) | bãi bỏ: Nghị định số 18/2021/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 134/2016/NĐ-CP ngày 01 tháng 9 năm 2016 của Chính phủ quy định chi  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=151157) | sửa đổi, bổ sung: Thông tư số 81/2018/TT-BTC Sửa đổi, bổ sung Thông tư số 83/2016/TT-BTC ngày 17/6/2016 của Bộ Tài chính hướng dẫn thực hiện ưu đãi đầu tư the (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=135988)</t>
+          <t>• 81/2018/TT-BTC — sửa đổi, bổ sung — hiệu lực 12/10/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=135988
+• 18/2021/NĐ-CP — bãi bỏ — hiệu lực 25/04/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=151157
+• Thông tư 20/2026/TT-BTC Quy định chi tiết một số điều của Luật Thuế thu nhập doanh nghiệp  — bãi bỏ — hiệu lực 10/03/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=6fb7dd80-59a6-11f1-a013-532655e6581a</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr"/>
@@ -1678,7 +1827,18 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 40/2026/NĐ-CP Quy định chi tiết một số điều của Luật Thủy lợi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=a0526ee0-791f-11f1-a7d3-6f8ab17b527d) | bãi bỏ: Nghị định số 32/2026/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định trong lĩnh vực chăn nuôi và thú y (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=aaff53a0-767f-11f1-a26c-15d47590a02f) | bãi bỏ: Nghị định số 39/2026/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 27/2019/NĐ-CP ngày 13 tháng 3 năm 2019 của Chính phủ quy định chi t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187831) | bãi bỏ: Nghị định số 23/2026/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định trong lĩnh vực tài nguyên nước (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186456) | bãi bỏ: Nghị định số 48/2026/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 08/2022/NĐ-CP ngày 10 tháng 01 năm 2022 của Chính phủ quy định chi  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187432) | thay thế: Nghị định số 43/2026/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định trong lĩnh vực bảo tồn thiên nhiên và đa dạng sinh học (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186739)</t>
+          <t>• 23/2026/NĐ-CP — bãi bỏ — hiệu lực 17/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186456
+• 32/2026/NĐ-CP — bãi bỏ — hiệu lực 21/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=aaff53a0-767f-11f1-a26c-15d47590a02f
+• 39/2026/NĐ-CP — bãi bỏ — hiệu lực 25/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187831
+• 40/2026/NĐ-CP — bãi bỏ — hiệu lực 25/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=a0526ee0-791f-11f1-a7d3-6f8ab17b527d
+• 43/2026/NĐ-CP — thay thế — hiệu lực 26/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186739
+• 48/2026/NĐ-CP — bãi bỏ — hiệu lực 29/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187432</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr"/>
@@ -1720,7 +1880,14 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 198/2025/NĐ-CP Quy định chi tiết một số điều và biện pháp thi hành Luật Phòng không nhân dân (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179783) | bãi bỏ: Nghị định số 222/2026/NĐ-CP về hoạt động bay (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=b6ab9020-8bbe-11f1-b2d0-6b22a52408be) | hợp nhất: Văn bản hợp nhất số 20/VBHN-BQP Quy định về quản lý độ cao chướng ngại vật hàng không và các trận địa quản lý, bảo vệ vùng trời tại Việt Nam (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179790) | sửa đổi, bổ sung: Nghị định số 101/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 32/2016/NĐ-CP ngày 06 tháng 5 năm 2016 của Chính phủ quy định về q (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=177726)</t>
+          <t>• 101/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 23/06/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=177726
+• 198/2025/NĐ-CP — bãi bỏ — hiệu lực 22/08/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179783
+• 222/2026/NĐ-CP — bãi bỏ — hiệu lực 01/07/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=b6ab9020-8bbe-11f1-b2d0-6b22a52408be
+• 20/VBHN-BQP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179790</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr"/>
@@ -1762,7 +1929,18 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 17/VBHN-BNNPTNT Quy định chi tiết thi hành một số điều của Luật Lâm nghiệp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166617) | hợp nhất: Văn bản hợp nhất số 24/VBHN-BNNPTNT Quy định chi tiết thi hành một số điều của Luật Lâm nghiệp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172573) | sửa đổi, bổ sung: Nghị định số 183/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 156/2018/NĐ-CP ngày 16 tháng 11 năm 2018 của Chính phủ quy định ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179099) | sửa đổi, bổ sung: Nghị định số 91/2024/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 156/2018/NĐ-CP ngày 16 tháng 11 năm 2018 của Chính phủ quy định chi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=168695) | sửa đổi, bổ sung: Nghị định số 227/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 156/2018/NĐ-CP ngày 16 tháng 11 năm 2018 của Chính phủ quy định ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186289) | thay thế: Nghị định số 58/2024/NĐ-CP Một số chính sách đầu tư trong lâm nghiệp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167508) | thay thế: Nghị định số 227/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 156/2018/NĐ-CP ngày 16 tháng 11 năm 2018 của Chính phủ quy định ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186289)</t>
+          <t>• 58/2024/NĐ-CP — thay thế — hiệu lực 15/07/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167508
+• 91/2024/NĐ-CP — sửa đổi, bổ sung — hiệu lực 18/07/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=168695
+• 183/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/08/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179099
+• 227/2025/NĐ-CP — sửa đổi, bổ sung, thay thế — hiệu lực 16/08/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186289
+• 17/VBHN-BNNPTNT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166617
+• 24/VBHN-BNNPTNT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172573</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr"/>
@@ -1804,7 +1982,22 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 92/2023/NĐ-CP Bãi bỏ một số văn bản quy phạm pháp luật của Chính phủ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164308) | hợp nhất: Văn bản hợp nhất số 951/VBHN-BTP Quy định chi tiết thi hành một số điều của Luật nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134587) | hợp nhất: Văn bản hợp nhất số 275/VBHN-BTP Quy định chi tiết thi hành một số điều của Luật Nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174653) | sửa đổi, bổ sung: Nghị định số 24/2019/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 19/2011/NĐ-CP ngày 21 tháng 3 năm 2011 của Chính phủ quy định chi t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134536) | sửa đổi, bổ sung: Nghị định số 18/2026/NĐ-CP Sửa đổi, bổ sung một số nghị định để cắt giảm, đơn giản hóa thủ tục hành chính, điều kiện kinh doanh thuộc phạm v (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187582) | sửa đổi, bổ sung: Nghị định số 06/2025/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định về nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174313) | sửa đổi, bổ sung: Nghị định số 114/2016/NĐ-CP Quy định lệ phí đăng ký nuôi con nuôi, lệ phí cấp giấy phép hoạt động của tổ chức con nuôi nước ngoài (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112160) | sửa đổi, bổ sung: Nghị định số 104/2022/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định liên quan đến việc nộp, xuất trình sổ hộ khẩu, sổ tạm trú giấy kh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167220)</t>
+          <t>• 114/2016/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112160
+• 24/2019/NĐ-CP — sửa đổi, bổ sung — hiệu lực 25/04/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134536
+• 104/2022/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167220
+• 92/2023/NĐ-CP — bãi bỏ — hiệu lực 19/12/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164308
+• 06/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 08/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174313
+• 18/2026/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187582
+• 275/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174653
+• 951/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=134587</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr"/>
@@ -1846,7 +2039,10 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 07/2021/TT-BVHTTDL quy định về tập huấn chuyên môn thể thao đối với người hướng dẫn tập luyện thể thao. (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=149703) | bãi bỏ: Thông tư số 21/2025/TT-BVHTTDL sửa đổi, bổ sung một số điều của các Thông tư có quy định thủ tục hành chính liên quan đến hoạt động sản xuất (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186002)</t>
+          <t>• 07/2021/TT-BVHTTDL — bãi bỏ — hiệu lực 01/12/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=149703
+• 21/2025/TT-BVHTTDL — bãi bỏ — hiệu lực 26/12/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186002</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr"/>
@@ -1888,7 +2084,10 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Nghị định số 42/2024/NĐ-CP Về hoạt động lấn biển (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167334) | sửa đổi, bổ sung: Nghị định số 104/2022/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định liên quan đến việc nộp, xuất trình sổ hộ khẩu, sổ tạm trú giấy kh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167220)</t>
+          <t>• 104/2022/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167220
+• 42/2024/NĐ-CP — sửa đổi, bổ sung — hiệu lực 16/04/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167334</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr"/>
@@ -1930,7 +2129,16 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 40/2024/TT-BGTVT Quy định về công tác phòng, chống, khắc phục hậu quả thiên tai trong lĩnh vực đường bộ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174157) | sửa đổi, bổ sung: Thông tư số 25/2024/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 50/2015/TT-BGTVT ngày 23 tháng 9 năm 2015 của Bộ trưởng Bộ Giao th (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=168214) | sửa đổi, bổ sung: Thông tư số 43/2021/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 03/2019/TT-BGTVT ngày 11 tháng 01 năm 2019 của Bộ trưởng Bộ Giao t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152588) | sửa đổi, bổ sung: Thông tư số 36/2020/TT-BGTVT Sửa đổi, bổ sung một số điều của các Thông tư quy định về chế độ báo cáo định kỳ trong lĩnh vực đường bộ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=145902) | sửa đổi, bổ sung: Thông tư số 22/2023/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 03/2019/TT-BGTVT ngày 11 tháng 01 năm 2019 của Bộ trưởng Bộ Giao t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=163042)</t>
+          <t>• 36/2020/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 15/02/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=145902
+• 43/2021/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 01/03/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152588
+• 22/2023/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 15/08/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=163042
+• 25/2024/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 01/08/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=168214
+• 40/2024/TT-BGTVT — bãi bỏ — hiệu lực 01/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174157</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr"/>
@@ -1972,7 +2180,14 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 14/2021/TT-BGTVT Bãi bỏ Điều 22 Thông tư số 31/2018/TT-BGTVT ngày 15 tháng 5 năm 2018 của Bộ trưởng Bộ Giao thông vận tải quy đị (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167004) | bãi bỏ: Thông tư số 34/2025/TT-BXD Quy định về quản lý, khai thác kết cấu hạ tầng đường sắt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=185678) | bãi bỏ: Thông tư số 01/2024/TT-BGTVT Quy định về việc kiểm tra chất lượng an toàn kỹ thuật và bảo vệ môi trường phương tiện giao thông đường sắt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166516) | bãi bỏ: Thông tư số 01/2022/TT-BGTVT Sửa đổi, bổ sung một số điều Thông tư số 29/2018/TT-BGTVT ngày 14 tháng 5 năm 2018 của Bộ trưởng Bộ Giao thông  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152592)</t>
+          <t>• 14/2021/TT-BGTVT — bãi bỏ — hiệu lực 01/08/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=167004
+• 01/2022/TT-BGTVT — bãi bỏ — hiệu lực 01/03/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152592
+• 01/2024/TT-BGTVT — bãi bỏ — hiệu lực 15/03/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166516
+• 34/2025/TT-BXD — bãi bỏ — hiệu lực 01/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=185678</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr"/>
@@ -2014,7 +2229,14 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 37/2016/TT-BCT Sửa đổi, bổ sung một số điều của Thông tư số 50/2014/TT-BCT ngày 15 tháng 12 năm 2014 của Bộ trưởng Bộ Công Thươn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=135507) | bãi bỏ: Thông tư số 25/2024/TT-BCT Bãi bỏ toàn bộ một số văn bản quy phạm pháp luật do Bộ trưởng Bộ Công Thương ban hành, liên tịch ban hành (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172166) | hợp nhất: Văn bản hợp nhất số 35/VBHN-BCT Quy định về quản lý nhiệm vụ khoa học và công nghệ của Bộ Công Thương (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141722) | sửa đổi, bổ sung: Thông tư số 42/2019/TT-BCT Sửa đổi, bổ sung một số quy định về chế độ báo cáo định kỳ tại các Thông tư do Bộ trưởng Bộ Công Thương ban hành  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139672)</t>
+          <t>• 37/2016/TT-BCT — bãi bỏ — hiệu lực 10/02/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=135507
+• 42/2019/TT-BCT — sửa đổi, bổ sung — hiệu lực 05/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139672
+• 25/2024/TT-BCT — bãi bỏ — hiệu lực 31/12/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172166
+• 35/VBHN-BCT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141722</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr"/>
@@ -2056,7 +2278,8 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>thay thế: Quyết định số 12/2005/QĐ-BGTVT Ban hành Điều lệ đường ngang (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=16270)</t>
+          <t>• 12/2005/QĐ-BGTVT — thay thế — hiệu lực 12/02/2005
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=16270</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr"/>
@@ -2098,7 +2321,18 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 01/2020/TT-BNNPTNT Quy định về chế độ báo cáo định kỳ thuộc phạm vi quản lý nhà nước của Bộ Nông nghiệp và Phát triển nông thôn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=142035) | bãi bỏ: Thông tư số 06/2022/TT-BNNPTNT Sửa đổi, bổ sung một số điều của các Thông tư quy định về kiểm dịch động vật, sản phẩm động vật thủy sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155158) | sửa đổi, bổ sung: Thông tư số 05/2025/TT-BNNMT Sửa đổi, bổ sung một số Thông tư trong lĩnh vực khai thác thuỷ sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178681) | sửa đổi, bổ sung: Thông tư số 01/2022/TT-BNNPTNT Sửa đổi, bổ sung một số Thông tư trong lĩnh vực thủy sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152678) | sửa đổi, bổ sung: Thông tư số 13/2020/TT-BNNPTNT Sửa đổi, bổ sung một số điều của Thông tư số 21/2018/TT-BNNPTNT ngày 15/11/2018 quy định ghi, nộp báo cáo, nh (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=144999) | thay thế: Thông tư số 81/2025/TT-BNNMT Quy định ghi, nộp báo cáo, nhật ký khai thác thủy sản; kiểm tra tàu cá và giám sát sản lượng thủy sản tại cảng  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186332)</t>
+          <t>• 01/2020/TT-BNNPTNT — bãi bỏ — hiệu lực 05/03/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=142035
+• 13/2020/TT-BNNPTNT — sửa đổi, bổ sung — hiệu lực 25/12/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=144999
+• 01/2022/TT-BNNPTNT — sửa đổi, bổ sung — hiệu lực 04/03/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152678
+• 06/2022/TT-BNNPTNT — bãi bỏ — hiệu lực 11/09/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155158
+• 05/2025/TT-BNNMT — sửa đổi, bổ sung — hiệu lực 18/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178681
+• 81/2025/TT-BNNMT — thay thế — hiệu lực 01/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186332</t>
         </is>
       </c>
       <c r="H35" s="8" t="inlineStr"/>
@@ -2140,7 +2374,16 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 63/2024/TT-NHNN Quy định về hồ sơ, thủ tục thu hồi Giấy phép và thanh lý tài sản của tổ chức tín dụng, chi nhánh ngân hàng nước  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174391) | hợp nhất: Văn bản hợp nhất số 29/VBHN-NHNN Quy định về trình tự, thủ tục thu hồi Giấy phép và thanh lý tài sản của tổ chức tín dụng, chi nhánh ngân hà (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=138117) | hợp nhất: Văn bản hợp nhất số 10/VBHN-NHNN Quy định về trình tự, thủ tục thu hồi Giấy phép và thanh lý tài sản của tổ chức tín dụng, chi nhánh ngân hà (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=145670) | sửa đổi, bổ sung: Thông tư số 11/2020/TT-NHNN Sửa đổi, bổ sung một số điều của Thông tư số 24/2017/TT-NHNN ngày 29 tháng 12 năm 2017 của Thống đốc Ngân hàng N (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=144726) | sửa đổi, bổ sung: Thông tư số 14/2019/TT-NHNN Sửa đổi, bổ sung một số điều tại các Thông tư có quy định về chế độ báo cáo định kỳ của Ngân hàng Nhà nước (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137583) | thay thế: Thông tư số 63/2024/TT-NHNN Quy định về hồ sơ, thủ tục thu hồi Giấy phép và thanh lý tài sản của tổ chức tín dụng, chi nhánh ngân hàng nước  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174391)</t>
+          <t>• 14/2019/TT-NHNN — sửa đổi, bổ sung — hiệu lực 15/10/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137583
+• 11/2020/TT-NHNN — sửa đổi, bổ sung — hiệu lực 17/12/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=144726
+• 63/2024/TT-NHNN — bãi bỏ, thay thế — hiệu lực 17/02/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174391
+• 10/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=145670
+• 29/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=138117</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr"/>
@@ -2182,7 +2425,10 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 4750/VBHN-BTP Quy định chế độ áp dụng biện pháp xử lý hành chính giáo dục tại xã, phường, đặc khu (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=180151) | sửa đổi, bổ sung: Nghị định số 190/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 118/2021/NĐ-CP ngày 23 tháng 12 năm 2021 của Chính phủ quy định ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179389)</t>
+          <t>• 190/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179389
+• 4750/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=180151</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr"/>
@@ -2224,7 +2470,12 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Nghị định số 18/2026/NĐ-CP Sửa đổi, bổ sung một số nghị định để cắt giảm, đơn giản hóa thủ tục hành chính, điều kiện kinh doanh thuộc phạm v (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187582) | sửa đổi, bổ sung: Nghị định số 112/2025/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định thuộc lĩnh vực bổ trợ tư pháp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178105) | thay thế: Nghị định số 112/2025/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định thuộc lĩnh vực bổ trợ tư pháp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178105) | thay thế: Nghị định số 65/2026/NĐ-CP Quy định chi tiết một số điều và biện pháp thi hành Luật Phục hồi, phá sản về Quản tài viên và hành nghề quản lý, (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187585)</t>
+          <t>• 112/2025/NĐ-CP — sửa đổi, bổ sung, thay thế — hiệu lực 29/05/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178105
+• 18/2026/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187582
+• 65/2026/NĐ-CP — thay thế — hiệu lực 01/03/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187585</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr"/>
@@ -2308,7 +2559,8 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Luật Tổ chức Toà án nhân dân số số: 34/2024/QH15 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170570)</t>
+          <t>• Luật Tổ chức Toà án nhân dân số số: 34/2024/QH15 — bãi bỏ — hiệu lực 01/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170570</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr"/>
@@ -2350,7 +2602,12 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 61/2026/NĐ-CP Quy định về danh mục, việc quản lý, sử dụng phương tiện, thiết bị kỹ thuật nghiệp vụ và quy trình thu thập, sử dụ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187090) | sửa đổi, bổ sung: Nghị định số 301/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 38/2024/NĐ-CP ngày 05 tháng 4 năm 2024 của Chính phủ quy định xử p (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186287) | thay thế: Nghị định số 246/2026/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực thủy sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=09419d10-79e6-11f1-b98d-21953d217c11)</t>
+          <t>• 301/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 17/11/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186287
+• 61/2026/NĐ-CP — bãi bỏ — hiệu lực 01/04/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187090
+• 246/2026/NĐ-CP — thay thế — hiệu lực 18/08/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=09419d10-79e6-11f1-b98d-21953d217c11</t>
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr"/>
@@ -2392,7 +2649,14 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 282/2025/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực an ninh, trật tự, an toàn xã hội; phòng, chống tệ nạn, xã hội (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=185254) | hợp nhất: Văn bản hợp nhất số 6545/VBHN-BTP Quy định xử phạt vi phạm hành chính trong lĩnh vực bổ trợ tư pháp; hành chính tư pháp; hôn nhân và gia đìn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=171730) | sửa đổi, bổ sung: Nghị định số 117/2024/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 82/2020/NĐ-CP ngày 15 tháng 7 năm 2020 của Chính phủ quy định xử p (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170131) | thay thế: Nghị định 109/2026/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực bổ trợ tư pháp; hành chính tư pháp; hôn nhân và gia đình; thi hà (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=0ae72df0-4247-11f1-9aef-8b444472143a)</t>
+          <t>• 117/2024/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/11/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170131
+• 282/2025/NĐ-CP — bãi bỏ — hiệu lực 15/12/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=185254
+• Nghị định 109/2026/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực bổ trợ tư pháp — thay thế — hiệu lực 18/05/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=0ae72df0-4247-11f1-9aef-8b444472143a
+• 6545/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=171730</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr"/>
@@ -2434,7 +2698,20 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 12/2024/TT-BTNMT Quy định chi tiết về đào tạo, bồi dưỡng, cập nhật kiến thức cho cá nhân hành nghề tư vấn định giá đất; khung ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=173538) | bãi bỏ: Thông tư số 26/2024/TT-BTNMT Quy định kỹ thuật về đo đạc lập bản đồ địa chính (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174271) | bãi bỏ: Thông tư số 27/2018/TT-BTNMT Quy định về thống kê, kiểm kê đất đai và lập bản đồ hiện trạng sử dụng đất (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133433) | bãi bỏ: Thông tư số 02/2023/TT-BTNMT Sửa đổi, bổ sung một số điều của Thông tư số 23/2014/TT-BTNMT ngày 19 tháng 5 năm 2014 của Bộ trưởng Bộ Tài ngu (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166137) | sửa đổi, bổ sung: Thông tư số 33/2017/TT-BTNMT Quy định chi tiết Nghị định số 01/2017/NĐ-CP ngày 06 tháng 01 năm 2017 của Chính phủ sửa đổi, bổ sung một số ng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=125567) | sửa đổi, bổ sung: Thông tư số 13/2019/TT-BTNMT Ban hành Quy định Định mức kinh tế - kỹ thuật thống kê, kiểm kê đất đai và lập bản đồ hiện trạng sử dụng đất (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137027) | sửa đổi, bổ sung: Thông tư số 09/2021/TT-BTNMT Sửa đổi, bổ sung một số điều của các Thông tư quy định chi tiết và hướng dẫn thi hành Luật Đất đai (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=149005)</t>
+          <t>• 33/2017/TT-BTNMT — sửa đổi, bổ sung — hiệu lực 05/12/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=125567
+• 27/2018/TT-BTNMT — bãi bỏ — hiệu lực 01/03/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133433
+• 13/2019/TT-BTNMT — sửa đổi, bổ sung — hiệu lực 23/09/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=137027
+• 09/2021/TT-BTNMT — sửa đổi, bổ sung — hiệu lực 01/09/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=149005
+• 02/2023/TT-BTNMT — bãi bỏ — hiệu lực 20/05/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166137
+• 12/2024/TT-BTNMT — bãi bỏ — hiệu lực 01/08/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=173538
+• 26/2024/TT-BTNMT — bãi bỏ — hiệu lực 15/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174271</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr"/>
@@ -2476,7 +2753,16 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Quyết định số 32/2023/QĐ-TTg Bãi bỏ toàn bộ hoặc một phần một số văn bản quy phạm pháp luật của Thủ tướng Chính phủ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166438) | bãi bỏ: Quyết định số 41/2026/QĐ-TTg Bãi bỏ một số văn bản quy phạm pháp luật của Thủ tướng Chính phủ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=4be348c0-9607-11f1-8d51-af7dccec1993) | bãi bỏ: Quyết định số 31/2015/QĐ-TTg Về định mức hành lý, tài sản di chuyển, quà biếu, quà tặng, hàng mẫu được miễn thuế, xét miễn thuế, không chịu  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=73839) | sửa đổi, bổ sung: Nghị định số 136/2007/NĐ-CP Về xuất cảnh, nhập cảnh của công dân Việt Nam (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=13615) | sửa đổi, bổ sung: Quyết định số 114/2001/QĐ-TTg Về việc sửa đổi, bổ sung một số điều của Quyết định số 210/1999/QĐ-TTg ngày 27 tháng 10 năm 1999 của Thủ tướng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=23253)</t>
+          <t>• 114/2001/QĐ-TTg — sửa đổi, bổ sung — hiệu lực 15/08/2001
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=23253
+• 136/2007/NĐ-CP — sửa đổi, bổ sung — hiệu lực 14/09/2007
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=13615
+• 31/2015/QĐ-TTg — bãi bỏ — hiệu lực 01/10/2015
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=73839
+• 32/2023/QĐ-TTg — bãi bỏ — hiệu lực 21/12/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166438
+• 41/2026/QĐ-TTg — bãi bỏ — hiệu lực 01/10/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=4be348c0-9607-11f1-8d51-af7dccec1993</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr"/>
@@ -2518,7 +2804,10 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>đình chỉ thi hành: Nghị định số 203/2026/NĐ-CP Quy định về thi hành án tử hình bằng tiêm thuốc độc (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=aac7bf60-7d02-11f1-844e-e9d0ea08e798) | sửa đổi, bổ sung: Nghị định số 184/2025/NĐ-CP Quy định phân định thẩm quyền khi tổ chức chính quyền địa phương 02 cấp và sửa đổi, bổ sung một số điều của các  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179825)</t>
+          <t>• 184/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179825
+• 203/2026/NĐ-CP — đình chỉ thi hành — hiệu lực 01/07/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=aac7bf60-7d02-11f1-844e-e9d0ea08e798</t>
         </is>
       </c>
       <c r="H45" s="8" t="inlineStr"/>
@@ -2560,7 +2849,8 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 221/2013/NĐ-CP Quy định chế độ áp dụng biện pháp xử lý hành chính đưa vào cơ sở cai nghiện bắt buộc (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32938)</t>
+          <t>• 221/2013/NĐ-CP — bãi bỏ — hiệu lực 15/02/2014
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32938</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr"/>
@@ -2602,7 +2892,12 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Thông tư số 07/2024/TT-BKHCN Sửa đổi, bổ sung một số điều tại các văn bản quy phạm pháp luật thuộc thẩm quyền của Bộ trưởng Bộ Khoa học và C (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170642) | sửa đổi, bổ sung: Thông tư số 13/2023/TT-BKHCN Bãi bỏ một số văn bản quy phạm pháp luật do Bộ trưởng Bộ Khoa học và Công nghệ ban hành, liên tịch ban hành (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162124) | thay thế: Thông tư số 54/2025/TT-BKHCN Quy định về hoạt động kiểm định, hiệu chuẩn, thử nghiệm phương tiện đo, chuẩn đo lường (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186195)</t>
+          <t>• 13/2023/TT-BKHCN — sửa đổi, bổ sung — hiệu lực 30/06/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162124
+• 07/2024/TT-BKHCN — sửa đổi, bổ sung — hiệu lực 22/11/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170642
+• 54/2025/TT-BKHCN — thay thế — hiệu lực 15/02/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186195</t>
         </is>
       </c>
       <c r="H47" s="8" t="inlineStr"/>
@@ -2644,7 +2939,10 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 11/VBHN-BXD Nghị định về xây dựng, quản lý, sử dụng nghĩa trang và cơ sở hỏa táng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=142413) | sửa đổi, bổ sung: Nghị định số 98/2019/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định thuộc lĩnh vực hạ tầng kỹ thuật (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=140187)</t>
+          <t>• 98/2019/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=140187
+• 11/VBHN-BXD — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=142413</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr"/>
@@ -2686,7 +2984,24 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 126/2020/NĐ-CP Quy định chi tiết một số điều của Luật Quản lý thuế (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=146459) | bãi bỏ: Nghị định số 181/2025/NĐ-CP Quy định chi tiết thi hành một số điều của Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187347) | bãi bỏ: Nghị định số 360/2025/NĐ-CP Quy định chi tiết thi hành một số điều của Luật Thuế tiêu thụ đặc biệt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186980) | hợp nhất: Văn bản hợp nhất số 31/VBHN-BTC Quy định chi tiết và hướng dẫn thi hành một số điều Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=158225) | hợp nhất: Văn bản hợp nhất số 18/VBHN-BTC Quy định chi tiết và hướng dẫn thi hành một số Điều của Luật thuế tiêu thụ đặc biệt và Luật sửa đổi, bổ sung (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118407) | hợp nhất: Văn bản hợp nhất số 16/VBHN-BTC Quy định về xử phạt vi phạm hành chính lĩnh vực về thuế và cưỡng chế thi hành quyết định hành chính thuế (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118404) | hợp nhất: Văn bản hợp nhất số 17/VBHN-BTC Quy định chi tiết và hướng dẫn thi hành một số điều Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118405) | hợp nhất: Văn bản hợp nhất số 19/VBHN-BTC Quy định chi tiết thi hành một số điều của Luật quản lý thuế và Luật sửa đổi, bổ sung một số điều của Luật q (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118408) | sửa đổi, bổ sung: Nghị định số 146/2017/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 100/2016/NĐ-CP ngày 01 tháng 7 năm 2016 và Nghị định số 12/2015/NĐ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=126410)</t>
+          <t>• 146/2017/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/02/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=126410
+• 126/2020/NĐ-CP — bãi bỏ — hiệu lực 05/12/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=146459
+• 181/2025/NĐ-CP — bãi bỏ — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187347
+• 360/2025/NĐ-CP — bãi bỏ — hiệu lực 01/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186980
+• 16/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118404
+• 17/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118405
+• 18/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118407
+• 19/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118408
+• 31/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=158225</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr"/>
@@ -2728,7 +3043,8 @@
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 01/2019/TT-BXD Bãi bỏ toàn bộ hoặc một phần một số văn bản quy phạm pháp luật do Bộ trưởng Bộ Xây dựng ban hành hoặc liên tịch b (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=136228)</t>
+          <t>• 01/2019/TT-BXD — bãi bỏ — hiệu lực 15/08/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=136228</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr"/>
@@ -2770,7 +3086,8 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Thông tư số 16/2026/TT-BXD Hướng dẫn xác định và quản lý các chi phí liên quan đến việc xây dựng, điều chỉnh chương trình, kế hoạch phát tri (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=5f662d30-8e47-11f1-8158-c1fa247e8bd5)</t>
+          <t>• 16/2026/TT-BXD — sửa đổi, bổ sung — hiệu lực 29/04/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=5f662d30-8e47-11f1-8158-c1fa247e8bd5</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr"/>
@@ -2812,7 +3129,10 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 74/2022/TT-BTC Quy định về hình thức, thời hạn thu, nộp, kê khai các khoản phí, lệ phí thuộc thẩm quyền quy định của Bộ Tài chín (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=158215) | sửa đổi, bổ sung: Thông tư số 06/2025/TT-BTC Sửa đổi, bổ sung một số điều của các Thông tư của Bộ trưởng Bộ Tài chính quy định về phí, lệ phí (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174853)</t>
+          <t>• 74/2022/TT-BTC — bãi bỏ — hiệu lực 22/12/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=158215
+• 06/2025/TT-BTC — sửa đổi, bổ sung — hiệu lực 10/03/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174853</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr"/>
@@ -2854,7 +3174,8 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>thay thế: Nghị định số 66/2014/NĐ-CP Quy định chi tiết, hướng dẫn thi hành một số điều của Luật Phòng, chống thiên tai (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=36766)</t>
+          <t>• 66/2014/NĐ-CP — thay thế — hiệu lực 20/08/2014
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=36766</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr"/>
@@ -2896,7 +3217,28 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 31/VBHN-BTC Quy định chi tiết và hướng dẫn thi hành một số điều Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=158225) | hợp nhất: Văn bản hợp nhất số 17/VBHN-BTC Quy định chi tiết và hướng dẫn thi hành một số điều Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118405) | hợp nhất: Văn bản hợp nhất số 13/VBHN-BTC Quy định chi tiết và hướng dẫn thi hành một số điều Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67827) | sửa đổi, bổ sung: Nghị định số 91/2014/NĐ-CP Sửa đổi, bổ sung một số điều tại các Nghị định quy định về thuế (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=37143) | sửa đổi, bổ sung: Nghị định số 100/2016/NĐ-CP Quy định chi tiết và hướng dẫn thi hành một số điều của Luật sửa đổi, bổ sung một số điều của Luật thuế giá trị  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112489) | sửa đổi, bổ sung: Nghị định số 49/2022/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 209/2013/NĐ-CP ngày 18 tháng 12 năm 2013 của Chính phủ quy định chi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155137) | sửa đổi, bổ sung: Nghị định số 146/2017/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 100/2016/NĐ-CP ngày 01 tháng 7 năm 2016 và Nghị định số 12/2015/NĐ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=126410) | sửa đổi, bổ sung: Nghị định số 12/2015/NĐ-CP Quy định chi tiết thi hành Luật sửa đổi, bổ sung một số điều của các Luật về thuế và sửa đổi, bổ sung một số điều (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=51578) | sửa đổi, bổ sung: Thông tư số 130/2016/TT-BTC Hướng dẫn thực hiện Nghị định số 100/2016/NĐ-CP ngày 01 tháng 7 năm 2016 của Chính phủ quy định chi tiết thi hàn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118086) | sửa đổi, bổ sung: Nghị định số 10/2017/NĐ-CP Ban hành Quy chế quản lý tài chính của Tập đoàn Điện lực Việt Nam và sửa đổi, bổ sung khoản 4 Điều 4 Nghị định số (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119077) | thay thế: Nghị định số 181/2025/NĐ-CP Quy định chi tiết thi hành một số điều của Luật Thuế giá trị gia tăng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187347)</t>
+          <t>• 91/2014/NĐ-CP — sửa đổi, bổ sung — hiệu lực 15/11/2014
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=37143
+• 12/2015/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2015
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=51578
+• 100/2016/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=112489
+• 130/2016/TT-BTC — sửa đổi, bổ sung — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118086
+• 10/2017/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/04/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119077
+• 146/2017/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/02/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=126410
+• 49/2022/NĐ-CP — sửa đổi, bổ sung — hiệu lực 12/09/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155137
+• 181/2025/NĐ-CP — thay thế — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187347
+• 13/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67827
+• 17/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=118405
+• 31/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=158225</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr"/>
@@ -2980,7 +3322,12 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 16/VBHN-BTC Quy định chi tiết phạm vi địa bàn hoạt động hải quan; trách nhiệm phối hợp trong phòng, chống buôn lậu, vận  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=129036) | sửa đổi, bổ sung: Nghị định số 153/2026/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 01/2015/NĐ-CP ngày 02 tháng 01 năm 2015 của Chính phủ quy định chi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=6f6eb4c0-7f30-11f1-87c0-45d4081ddc83) | sửa đổi, bổ sung: Nghị định số 12/2018/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 01/2015/NĐ-CP ngày 02 tháng 01 năm 2015 của Chính phủ quy định chi  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=128877)</t>
+          <t>• 12/2018/NĐ-CP — sửa đổi, bổ sung — hiệu lực 10/03/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=128877
+• 153/2026/NĐ-CP — sửa đổi, bổ sung — hiệu lực 05/07/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=6f6eb4c0-7f30-11f1-87c0-45d4081ddc83
+• 16/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=129036</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr"/>
@@ -3022,7 +3369,10 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 364/VBHN-BVHTTDL Nghị định (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=b14c2470-9bb1-11f1-90e8-e7dd3137bfa4) | sửa đổi, bổ sung: Nghị định số 129/2021/NĐ-CP sửa đổi, bổ sung một số điều của các Nghị định quy định xử phạt vi phạm hành chính trong lĩnh vực du lịch; thể t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155691)</t>
+          <t>• 129/2021/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155691
+• 364/VBHN-BVHTTDL — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=b14c2470-9bb1-11f1-90e8-e7dd3137bfa4</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr"/>
@@ -3064,7 +3414,14 @@
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 02/VBHN-BKHCN Quy định về xử phạt vi phạm hành chính trong lĩnh vực tiêu chuẩn, đo lường, chất lượng sản phẩm, hàng hóa (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=154195) | sửa đổi, bổ sung: Nghị định số 126/2021/NĐ-CP Sửa đổi, bổ sung một số điều của các nghị định quy định xử phạt vi phạm hành chính trong lĩnh vực sở hữu công ng (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=154199) | sửa đổi, bổ sung: Nghị định số 42/2019/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực thủy sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=135367) | sửa đổi, bổ sung: Nghị định số 106/2025/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực phòng cháy, chữa cháy và cứu nạn, cứu hộ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=177735)</t>
+          <t>• 42/2019/NĐ-CP — sửa đổi, bổ sung — hiệu lực 05/07/2019
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=135367
+• 126/2021/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=154199
+• 106/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=177735
+• 02/VBHN-BKHCN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=154195</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr"/>
@@ -3106,7 +3463,16 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 40/2024/TT-BGTVT Quy định về công tác phòng, chống, khắc phục hậu quả thiên tai trong lĩnh vực đường bộ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174157) | sửa đổi, bổ sung: Thông tư số 25/2024/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 50/2015/TT-BGTVT ngày 23 tháng 9 năm 2015 của Bộ trưởng Bộ Giao th (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=168214) | sửa đổi, bổ sung: Thông tư số 43/2021/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 03/2019/TT-BGTVT ngày 11 tháng 01 năm 2019 của Bộ trưởng Bộ Giao t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152588) | sửa đổi, bổ sung: Thông tư số 36/2020/TT-BGTVT Sửa đổi, bổ sung một số điều của các Thông tư quy định về chế độ báo cáo định kỳ trong lĩnh vực đường bộ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=145902) | sửa đổi, bổ sung: Thông tư số 22/2023/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 03/2019/TT-BGTVT ngày 11 tháng 01 năm 2019 của Bộ trưởng Bộ Giao t (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=163042)</t>
+          <t>• 36/2020/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 15/02/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=145902
+• 43/2021/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 01/03/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152588
+• 22/2023/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 15/08/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=163042
+• 25/2024/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 01/08/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=168214
+• 40/2024/TT-BGTVT — bãi bỏ — hiệu lực 01/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=174157</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr"/>
@@ -3148,7 +3514,18 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: LUẬT THI HÀNH TẠM GIỮ, TẠM GIAM VÀ CẤM ĐI KHỎI NƠI CƯ TRÚ SỐ 128/2025/QH15 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186570) | sửa đổi, bổ sung: Luật Tư pháp người chưa thành niên số 59/2024/QH15 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=175425) | sửa đổi, bổ sung: Luật Giám định tư pháp số 105/2025/QH15 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187758) | sửa đổi, bổ sung: Luật sửa đổi, bổ sung một số điều của Bộ luật Tố tụng hình sự số 02/2021/QH15 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=153151) | sửa đổi, bổ sung: Luật sửa đổi, bổ sung một số điều của Luật Hải quan số 11/2026/QH16 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=9e4921a0-a2b1-11f1-8b6e-45ba51c9efb5) | sửa đổi, bổ sung: Luật Tổ chức Toà án nhân dân số số: 34/2024/QH15 (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170570)</t>
+          <t>• Luật sửa đổi, bổ sung một số điều của Bộ luật Tố tụng hình sự số 02/2021/QH15 — sửa đổi, bổ sung — hiệu lực 01/12/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=153151
+• Luật Tổ chức Toà án nhân dân số số: 34/2024/QH15 — sửa đổi, bổ sung — hiệu lực 01/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=170570
+• 59/2024/QH15 — sửa đổi, bổ sung — hiệu lực 01/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=175425
+• 105/2025/QH15 — sửa đổi, bổ sung — hiệu lực 01/05/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=187758
+• LUẬT THI HÀNH TẠM GIỮ, TẠM GIAM VÀ CẤM ĐI KHỎI NƠI CƯ TRÚ SỐ 128/2025/QH15 — sửa đổi, bổ sung — hiệu lực 01/07/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186570
+• Luật sửa đổi, bổ sung một số điều của Luật Hải quan số 11/2026/QH16 — sửa đổi, bổ sung — hiệu lực 01/03/2027
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=9e4921a0-a2b1-11f1-8b6e-45ba51c9efb5</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr"/>
@@ -3190,7 +3567,10 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 12/2025/TT-BTP Ban hành, hướng dẫn sử dụng, quản lý mẫu sổ quốc tịch và mẫu giấy tờ về quốc tịch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186318) | hợp nhất: Văn bản hợp nhất số 4101/VBHN-BTP Ban hành, hướng dẫn sử dụng, quản lý mẫu sổ quốc tịch và mẫu giấy tờ về quốc tịch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169236)</t>
+          <t>• 12/2025/TT-BTP — bãi bỏ — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186318
+• 4101/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=169236</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr"/>
@@ -3232,7 +3612,8 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>thay thế: Nghị định số 136/2006/NĐ-CP Quy định chi tiết và hướng dẫn thi hành một số điều của Luật Khiếu nại, tố cáo và các Luật sửa đổi, bổ sung một  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=14979)</t>
+          <t>• 136/2006/NĐ-CP — thay thế — hiệu lực 09/12/2006
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=14979</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr"/>
@@ -3274,7 +3655,10 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Nghị định số 09/2005/NĐ-CP Về việc quy định xử phạt vi phạm hành chính trong lĩnh vực giao thông đường thuỷ nội địa (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=18507) | sửa đổi, bổ sung: Nghị định số 77/1998/NĐ-CP Về sửa đổi, bổ sung một số điều của Nghị định số 40/CP ngày 5/7/1996 của Chính phủ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=7469)</t>
+          <t>• 77/1998/NĐ-CP — sửa đổi, bổ sung — hiệu lực 11/10/1998
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=7469
+• 09/2005/NĐ-CP — sửa đổi, bổ sung — hiệu lực 24/02/2005
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=18507</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr"/>
@@ -3316,7 +3700,18 @@
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 06/VBHN-BTC Hướng dẫn thi hành một số điều của nghị định số 45/2007/NĐ-CP ngày 27 tháng 3 năm 2007 của Chính phủ quy địn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67761) | hợp nhất: Văn bản hợp nhất số 06/VBHN-BTC Hướng dẫn thi hành một số điều của Nghị định số 45/2007/NĐ-CP ngày 27 tháng 3 năm 2007 của Chính phủ quy địn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111472) | sửa đổi, bổ sung: Thông tư số 124/2012/TT-BTC Hướng dẫn thi hành một số điều của Nghị định số 45/2007/NĐ-CP ngày 27 tháng 3 năm 2007 của Chính phủ quy định ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67760) | sửa đổi, bổ sung: Thông tư số 194/2014/TT-BTC Sửa đổi, bổ sung một số điều của Thông tư số 124/2012/TT-BTC ngày 30/7/2012 của Bộ Tài chính hướng dẫn thi hành  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67756) | thay thế: Thông tư số 50/2017/TT-BTC Hướng dẫn thi hành Nghị định số 73/2016/NĐ-CP ngày 01 tháng 7 năm 2016 của Chính phủ quy đinh chi tiết thi hành L (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122601) | thay thế: Thông tư số 50/2017/TT-BTC Hướng dẫn thi hành Nghị định số 73/2016/NĐ-CP ngày 01 tháng 7 năm 2016 của Chính phủ quy định chi tiết thi hành L (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122433)</t>
+          <t>• 124/2012/TT-BTC — sửa đổi, bổ sung — hiệu lực 01/10/2012
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67760
+• 194/2014/TT-BTC — sửa đổi, bổ sung — hiệu lực 01/02/2015
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67756
+• 50/2017/TT-BTC — thay thế — hiệu lực 01/07/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122433
+• 50/2017/TT-BTC — thay thế — hiệu lực 01/07/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122601
+• 06/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111472
+• 06/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=67761</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr"/>
@@ -3358,7 +3753,14 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 09/VBHN-BTC Quy định xử phạt vi phạm hành chính trong lĩnh vực chứng khoán và thị trường chứng khoán (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=156570) | hợp nhất: Văn bản hợp nhất số 17/VBHN-BTC Nghị định số 156/2020/NĐ-CP Quy định xử phạt vi phạm hành chính trong lĩnh vực chứng khoán và thị trường chứ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=f69936f0-6937-11f1-a48d-29bc6b0fd706) | sửa đổi, bổ sung: Nghị định số 128/2021/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 156/2020/NĐ-CP ngày 31 tháng 12 năm 2020 của Chính phủ quy định xử (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152529) | sửa đổi, bổ sung: Nghị định số 306/2025/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 156/2020/NĐ-CP ngày 31 tháng 12 năm 2020 của Chính phủ quy định xử (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186388)</t>
+          <t>• 128/2021/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/01/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152529
+• 306/2025/NĐ-CP — sửa đổi, bổ sung — hiệu lực 09/01/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186388
+• 09/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=156570
+• 17/VBHN-BTC — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=f69936f0-6937-11f1-a48d-29bc6b0fd706</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr"/>
@@ -3400,7 +3802,10 @@
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Thông tư số 17/2023/TT-BGTVT Sửa đổi, bổ sung một số điều của Thông tư số 40/2016/TT-BGTVT ngày 7 tháng 12 năm 2016 của Bộ trưởng Bộ Giao th (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=161666) | sửa đổi, bổ sung: Thông tư số 16/2022/TT-BGTVT Sửa đổi, bổ sung một số điều của các Thông tư trong lĩnh vực đăng kiểm (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=154915)</t>
+          <t>• 16/2022/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 15/08/2022
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=154915
+• 17/2023/TT-BGTVT — sửa đổi, bổ sung — hiệu lực 15/08/2023
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=161666</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr"/>
@@ -3442,7 +3847,10 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 137/2024/NĐ-CP Quy định về giao dịch điện tử của cơ quan nhà nước và hệ thống thông tin phục vụ giao dịch điện tử (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=171147) | bãi bỏ: Nghị định số 47/2024/NĐ-CP Quy định về Danh mục Cơ sở dữ liệu quốc gia; việc xây dựng, cập nhật, duy trì, khai khác và sử dụng cơ sở dữ liệu (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166966)</t>
+          <t>• 47/2024/NĐ-CP — bãi bỏ — hiệu lực 09/05/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=166966
+• 137/2024/NĐ-CP — bãi bỏ — hiệu lực 23/10/2024
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=171147</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr"/>
@@ -3484,7 +3892,10 @@
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 07/2017/TT-BLĐTBXH Quy định chế độlàm việc của nhà giáo giáo dục nghề nghiệp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119515) | bãi bỏ: Thông tư số 08/2017/TT-BLĐTBXH Quy định chuẩn về chuyên môn, nghiệp vụ của nhà giáo giáo dục nghề nghiệp (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119519)</t>
+          <t>• 08/2017/TT-BLĐTBXH — bãi bỏ — hiệu lực 01/05/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119519
+• 07/2017/TT-BLĐTBXH — bãi bỏ — hiệu lực 01/07/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119515</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr"/>
@@ -3526,7 +3937,10 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 27/2019/TT-BLĐTBXH Ban hành danh mục thiết bị đào tạo tối thiểu trình độ trung cấp, trình độ cao đẳng cho một số nghề thuộc nhóm (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141640) | bãi bỏ: Thông tư số 26/2019/TT-BLĐTBXH Ban hành danh mục thiết bị đào tạo tối thiểu trình độ trung cấp, trình độ cao đẳng cho một số nghề thuộc nhóm (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141638)</t>
+          <t>• 26/2019/TT-BLĐTBXH — bãi bỏ — hiệu lực 09/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141638
+• 27/2019/TT-BLĐTBXH — bãi bỏ — hiệu lực 09/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141640</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr"/>
@@ -3568,7 +3982,8 @@
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Thông tư số 128/2013/TT-BTC Quy định về thủ tục hải quan; kiểm tra, giám sát hải quan; thuế xuất khẩu, thuế nhập khẩu và quản lý thuế đối vớ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32604) | thay thế: Thông tư số 128/2013/TT-BTC Quy định về thủ tục hải quan; kiểm tra, giám sát hải quan; thuế xuất khẩu, thuế nhập khẩu và quản lý thuế đối vớ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32604)</t>
+          <t>• 128/2013/TT-BTC — bãi bỏ, thay thế — hiệu lực 01/11/2013
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32604</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr"/>
@@ -3610,7 +4025,20 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 34/VBHN-NHNN Quy định về phát hành kỳ phiếu, tín phiếu, chứng chỉ tiền gửi, trái phiếu trong nước của tổ chức tín dụng,  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111763) | hợp nhất: Văn bản hợp nhất số 14/VBHN-NHNN Quy định về phát hành kỳ phiếu, tín phiếu, chứng chỉ tiền gửi, trái phiếu trong nước của tổ chức tín dụng,  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=102033) | hợp nhất: Văn bản hợp nhất số 05/VBHN-NHNN Quy định về phát hành kỳ phiếu, tín phiếu, chứng chỉ tiền gửi, trái phiếu trong nước của tổ chức tín dụng,  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=140654) | sửa đổi, bổ sung: Thông tư số 16/2016/TT-NHNN Sửa đổi, bổ sung một số điều của Thông tư số 34/2013/TT-NHNN ngày 31 tháng 12 năm 2013 của Thống đốc Ngân hàng N (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111664) | sửa đổi, bổ sung: Thông tư số 29/2015/TT-NHNN Sửa đổi, bổ sung một số văn bản quy phạm pháp luật của Ngân hàng Nhà nước Việt Nam quy định về thành phần hồ sơ  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=96046) | sửa đổi, bổ sung: Thông tư số 33/2019/TT-NHNN Sửa đổi, bổ sung một số điều của Thông tư số 34/2013/TT-NHNN ngày 31 tháng 12 năm 2013 của Thống đốc Ngân hàng N (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139893) | thay thế: Thông tư số 01/2021/TT-NHNN Quy định về phát hành kỳ phiếu, tín phiếu, chứng chỉ tiền gửi, trái phiếu trong nước của tổ chức tín dụng, chi n (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147126)</t>
+          <t>• 29/2015/TT-NHNN — sửa đổi, bổ sung — hiệu lực 08/02/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=96046
+• 16/2016/TT-NHNN — sửa đổi, bổ sung — hiệu lực 01/07/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111664
+• 33/2019/TT-NHNN — sửa đổi, bổ sung — hiệu lực 19/02/2020
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139893
+• 01/2021/TT-NHNN — thay thế — hiệu lực 17/05/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147126
+• 05/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=140654
+• 14/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=102033
+• 34/VBHN-NHNN — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111763</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr"/>
@@ -3652,7 +4080,16 @@
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 123/2015/NĐ-CP Quy định chi tiết một số điều và biện pháp thi hành Luật Hộ tịch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=92897) | bãi bỏ: Nghị định số 19/2011/NĐ-CP Quy định chi tiết thi hành một số điều của Luật Nuôi con nuôi (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=26222) | hợp nhất: Văn bản hợp nhất số 8013/VBHN-BTP Về đăng ký và quản lý hộ tịch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32721) | hợp nhất: Văn bản hợp nhất số 8013/VBHN-BTP Về đăng ký và quản lý hộ tịch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32948) | sửa đổi, bổ sung: Nghị định số 06/2012/NĐ-CP Sửa đổi, bổ sung một số điều của các Nghị định về hộ tịch, hôn nhân và gia đình và chứng thực (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=27159)</t>
+          <t>• 19/2011/NĐ-CP — bãi bỏ — hiệu lực 08/05/2011
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=26222
+• 06/2012/NĐ-CP — sửa đổi, bổ sung — hiệu lực 01/04/2012
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=27159
+• 123/2015/NĐ-CP — bãi bỏ — hiệu lực 01/01/2016
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=92897
+• 8013/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32721
+• 8013/VBHN-BTP — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32948</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr"/>
@@ -3694,7 +4131,22 @@
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 04/VBHN-BNNPTNT hợp nhất Thông tư quy định về kiểm tra, chứng nhận an toàn thực phẩm thủy sản xuất khẩu. (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=136878) | hợp nhất: Văn bản hợp nhất số 02/VBHN-BNNPTNT Quy định về kiểm tra, chứng nhận an toàn thực phẩm thủy sản xuất khẩu (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=159656) | hợp nhất: Văn bản hợp nhất số 32/VBHN-BNNPTNT Quy định về thẩm định, chứng nhận an toàn thực phẩm thủy sản xuất khẩu (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172683) | sửa đổi, bổ sung: Thông tư số 02/2017/TT-BNNPTNT Sửa đổi, bổ sung một số điều tại thông tư số 48/2013/TT-BNNPTNT ngày 12/11/2013 quy định về kiểm tra, chứng n (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122443) | sửa đổi, bổ sung: Thông tư số 16/2018/TT-BNNPTNT sửa đổi, bổ sung một số điều của Thông tư số 48/2013/TT-BNNPTNT ngày 12/11/2013 của Bộ trưởng Bộ Nông nghiệp  (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=132279) | sửa đổi, bổ sung: Thông tư số 17/2025/TT-BNNMT Quy định về phân cấp quản lý nhà nước trong lĩnh vực quản lý chất lượng nông lâm sản và thủy sản (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178667) | sửa đổi, bổ sung: Thông tư số 17/2024/TT-BNNPTNT Sửa đổi, bổ sung một số Thông tư quy định thẩm định, chứng nhận cơ sở sản xuất, kinh doanh thực phẩm nông, lâ (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172685) | thay thế: Thông tư số 80/2025/TT-BNNMT Quy định về thẩm định, chứng nhận an toàn thực phẩm thủy sản xuất khẩu (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186338)</t>
+          <t>• 02/2017/TT-BNNPTNT — sửa đổi, bổ sung — hiệu lực 30/03/2017
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122443
+• 16/2018/TT-BNNPTNT — sửa đổi, bổ sung — hiệu lực 13/12/2018
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=132279
+• 17/2024/TT-BNNPTNT — sửa đổi, bổ sung — hiệu lực 15/01/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172685
+• 17/2025/TT-BNNMT — sửa đổi, bổ sung — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178667
+• 80/2025/TT-BNNMT — thay thế — hiệu lực 02/02/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186338
+• 02/VBHN-BNNPTNT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=159656
+• 04/VBHN-BNNPTNT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=136878
+• 32/VBHN-BNNPTNT — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172683</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr"/>
@@ -3736,7 +4188,10 @@
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>bãi bỏ: Nghị định số 118/2025/NĐ-CP Về thực hiện thủ tục hành chính theo cơ chế một cửa, một cửa liên thông tại Bộ phận Một cửa và Cổng Dịch vụ công (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178283) | sửa đổi, bổ sung: Nghị định số 107/2021/NĐ-CP Sửa đổi Nghị định 61/2018/NĐ-CP về thực hiện cơ chế một cửa, một cửa liên thông trong giải quyết thủ tục hành ch (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162258)</t>
+          <t>• 107/2021/NĐ-CP — sửa đổi, bổ sung — hiệu lực 06/12/2021
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=162258
+• 118/2025/NĐ-CP — bãi bỏ — hiệu lực 01/07/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=178283</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr"/>
@@ -3778,7 +4233,10 @@
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>hợp nhất: Văn bản hợp nhất số 40 /VBHN-BCT Thông tư Quy định điều độ, vận hành, thao tác, xử lý sự cố, khởi động đen và khôi phục hệ thống điện quốc g (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=180482) | sửa đổi, bổ sung: Thông tư số 46/2025/TT-BCT Sửa đổi, bổ sung một số điều của Thông tư số 04/2025/TT-BCT ngày 01 tháng 02 năm 2025 của Bộ trưởng Bộ Công Thươn (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=180486)</t>
+          <t>• 46/2025/TT-BCT — sửa đổi, bổ sung — hiệu lực 22/09/2025
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=180486
+• Văn bản hợp nhất số 40 /VBHN-BCT Thông tư Quy định điều độ, vận hành, thao tác, xử lý sự c — văn bản hợp nhất, chỉ để tham khảo lời văn
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=180482</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr"/>
@@ -3820,7 +4278,8 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>sửa đổi, bổ sung: Nghị định 69/2026/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 106/2025/NĐ-CP ngày 15 tháng 5 năm 2025 của Chính phủ quy định xử phạt (https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=e23574c0-4c1e-11f1-b4dc-a19f4e8a4d2c)</t>
+          <t>• Nghị định 69/2026/NĐ-CP Sửa đổi, bổ sung một số điều của Nghị định số 106/2025/NĐ-CP ngày  — sửa đổi, bổ sung — hiệu lực 20/04/2026
+  https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=e23574c0-4c1e-11f1-b4dc-a19f4e8a4d2c</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr"/>

</xml_diff>